<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-03 Le pique-nique de la pente
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-03.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-03.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut pique-niquer le biscuit sur la pente. La gourde pique, le chapeau est trop haut. Il enveloppe, range, croque dans l'herbe.</t>
+          <t>Nino veut croquer le biscuit chaud sur la pente, tout de suite. Il part les bras pleins : la gourde tombe. Il refuse de foncer. L'éclat de marche libère la sangle. Le sac ferme. Le biscuit croque dans l'herbe, l'éclat pâle sur le rouge.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le vent de la pente plie l'herbe. L'herbe sent le foin, tout sec. La maison de bois craque un peu. Une casserole chuchote dans la cuisine. Ça sent le biscuit tout chaud. Une vapeur légère danse près du four. Dehors, une pierre grise chauffe déjà. Un oiseau de montagne crie, tout haut. Nino, le biscuit est prêt. On le mange dehors ? Oui, sur la pente. Un pique-nique, tout petit. En ce moment, Nino s'accroupit. Le sac rouge est par terre. La sangle est lisse, un peu froide. Il est rouge, maman. Oui, c'est le tien. Le goûter d'abord, encore chaud. Nino prend le petit paquet. Le papier fait un bruit doux. Ça sent encore le biscuit. Je le mange maintenant ? Plus tard, dans l'herbe. D'abord, dans le sac. Nino pose le goûter dedans. Prends aussi de l'eau. Nino prend la gourde verte. Elle est trop froide pour ses doigts. Aïe, elle pique. Enveloppe-la dans le linge. Un linge à carreaux attend sur la table. Nino l'enroule autour de l'eau. Le froid s'en va un peu. C'est mieux. Il pose la gourde dans le sac. Où est le chapeau ? Le crochet du bas est vide. Le chapeau est trop haut. Je te le tends ? Oui, s'il te plaît.</t>
+          <t>Dans le chalet, une casserole chuchote. Le vent de la pente lui répond. Il glisse sous la porte, frais. Il touche la première marche. Un éclat de marche brille, pâle. Nino le voit, sans savoir. L'herbe dehors sent le foin. La maison de bois craque. Ça sent le biscuit, tout chaud. Une vapeur danse près du four. Dehors, une pierre grise chauffe. Un oiseau de montagne crie, haut. Nino, le biscuit est prêt. On le mange dehors, tout de suite ? Oui, sur la pente. Un pique-nique, tout petit. En ce moment, Nino saisit le paquet. Le papier est tiède sous les doigts. Je le porte, maman. Pas besoin du sac. Il prend aussi la gourde verte. Elle pique, trop froide. Aïe ! Il court vers la porte, les bras pleins. Le vent pousse le battant. Le paquet glisse. La gourde tombe sur le bois. Patatras. Oh. Le biscuit roule vers le seuil. Nino le rattrape, les joues chaudes. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. Tu voulais partir tout de suite ? Le biscuit va refroidir. Maman s'accroupit, à sa hauteur. Où le biscuit voyage-t-il mieux ? Dans mes mains. Le papier se froisse, trop lâche. Le sac rouge attend par terre. La sangle est lisse, un peu froide. Il est rouge. Oui, c'est le tien. Nino pose le biscuit dedans. Le papier se tait. L'eau aussi. Un linge à carreaux attend. Nino l'enroule autour de l'eau. C'est moins froid. Il glisse l'eau dans le sac. Où est le chapeau ? Le crochet du bas est vide. Le chapeau est trop haut.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le vent de la pente plie l'herbe. L'herbe sent le foin, tout sec. La maison de bois craque un peu. Une casserole chuchote dans la cuisine. Ça sent le biscuit tout chaud. Une vapeur légère danse près du four. Dehors, une pierre grise chauffe déjà. Un oiseau de montagne crie, tout haut. Nino, le biscuit est prêt. On le mange dehors ? Oui, sur la pente. Un pique-nique, tout petit. En ce moment, Nino s'accroupit. Le sac rouge est par terre. La sangle est lisse, un peu froide. Il est rouge, maman. Oui, c'est le tien. Le goûter d'abord, encore chaud. Nino prend le petit paquet. Le papier fait un bruit doux. Ça sent encore le biscuit. Je le mange maintenant ? Plus tard, dans l'herbe. D'abord, dans le sac. Nino pose le goûter dedans. Prends aussi de l'eau. Nino prend la gourde verte. Elle est trop froide pour ses doigts. Aïe, elle pique. Enveloppe-la dans le linge. Un linge à carreaux attend sur la table. Nino l'enroule autour de l'eau. Le froid s'en va un peu. C'est mieux. Il pose la gourde dans le sac. Où est le chapeau ? Le crochet du bas est vide. Le chapeau est trop haut. Je te le tends ? Oui, s'il te plaît.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans le chalet, une casserole chuchote. Le vent de la pente lui répond. Il glisse sous la porte, frais. Il touche la première marche. Un &lt;emphasis level="moderate"&gt;éclat de marche&lt;/emphasis&gt; brille, pâle. Nino le voit, sans savoir. L'herbe dehors sent le foin. La maison de bois craque. Ça sent le biscuit, tout chaud. Une vapeur danse près du four. Dehors, une pierre grise chauffe. Un oiseau de montagne crie, haut. Nino, le biscuit est prêt. On le mange dehors, tout de suite ? Oui, sur la pente. Un pique-nique, tout petit. En ce moment, Nino saisit le paquet. Le papier est tiède sous les doigts. Je le porte, maman. Pas besoin du sac. Il prend aussi la gourde verte. Elle pique, trop froide. Aïe ! Il court vers la porte, les bras pleins. Le vent pousse le battant. Le paquet glisse. La gourde tombe sur le bois. Patatras. Oh. Le biscuit roule vers le seuil. Nino le rattrape, les joues chaudes. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. Tu voulais partir tout de suite ? Le biscuit va refroidir. Maman s'accroupit, à sa hauteur. Où le biscuit voyage-t-il mieux ? Dans mes mains. Le papier se froisse, trop lâche. Le sac rouge attend par terre. La sangle est lisse, un peu froide. Il est rouge. Oui, c'est le tien. Nino pose le biscuit dedans. Le papier se tait. L'eau aussi. Un linge à carreaux attend. Nino l'enroule autour de l'eau. C'est moins froid. Il glisse l'eau dans le sac. Où est le chapeau ? Le crochet du bas est vide. Le chapeau est trop haut.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est le matin. Dounia est dans l'entrée. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est par terre. Il est rouge. Maman est là, près de Dounia. Maman est l'adulte. Maman dit : la gourde, le chapeau, le goûter. Dounia écoute. Dounia voit la gourde verte. Elle la prend. Elle la met dans le sac. Dounia voit le chapeau souple. Elle le prend. Elle le met dans le sac. Dounia voit le petit goûter. Elle le prend. Elle le met dans le sac. Dounia appuie sur la fermeture. Ça fait zzz. Le sac est fermé. Dounia a mis ce que l'adulte a dit. Maman pose la main sur le sac. Maman dit : merci Dounia. Le sac est prêt.&lt;/slow&gt; [pause]</t>
+          <t>Dans le chalet, une casserole chuchote. Le vent de la pente lui répond. Il glisse sous la porte, frais. Il touche la première marche. Un &lt;emphasis&gt;éclat de marche&lt;/emphasis&gt; brille, pâle. Nino le voit, sans savoir. L'herbe dehors sent le foin. La maison de bois craque. Ça sent le biscuit, tout chaud. Une vapeur danse près du four. Dehors, une pierre grise chauffe. Un oiseau de montagne crie, haut. Nino, le biscuit est prêt. On le mange dehors, tout de suite ? Oui, sur la pente. Un pique-nique, tout petit. En ce moment, Nino saisit le paquet. Le papier est tiède sous les doigts. Je le porte, maman. Pas besoin du sac. Il prend aussi la gourde verte. Elle pique, trop froide. Aïe ! Il court vers la porte, les bras pleins. Le vent pousse le battant. Le paquet glisse. La gourde tombe sur le bois. Patatras. Oh. Le biscuit roule vers le seuil. Nino le rattrape, les joues chaudes. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. Tu voulais partir tout de suite ? Le biscuit va refroidir. Maman s'accroupit, à sa hauteur. Où le biscuit voyage-t-il mieux ? Dans mes mains. Le papier se froisse, trop lâche. Le sac rouge attend par terre. La sangle est lisse, un peu froide. Il est rouge. Oui, c'est le tien. Nino pose le biscuit dedans. Le papier se tait. L'eau aussi. Un linge à carreaux attend. Nino l'enroule autour de l'eau. C'est moins froid. Il glisse l'eau dans le sac. Où est le chapeau ? Le crochet du bas est vide. Le chapeau est trop haut. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de marche</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,51 +1319,73 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=ouvrir_le_monde; emotion=impatience; intensite=2; destinataire=enfant; sous_texte=le biscuit veut sortir tout de suite; tempo=naturel; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le vent de la pente plie l'herbe.
-narrateur|L'herbe sent le foin, tout sec.
-narrateur|La maison de bois craque un peu.
-narrateur|Une casserole chuchote dans la cuisine.
-narrateur|Ça sent le biscuit tout chaud.
-narrateur|Une vapeur légère danse près du four.
-narrateur|Dehors, une pierre grise chauffe déjà.
-narrateur|Un oiseau de montagne crie, tout haut.
+          <t>narrateur|Dans le chalet, une casserole chuchote.
+narrateur|Le vent de la pente lui répond.
+narrateur|Il glisse sous la porte, frais.
+narrateur|Il touche la première marche.
+narrateur|Un éclat de marche brille, pâle.
+narrateur|Nino le voit, sans savoir.
+narrateur|L'herbe dehors sent le foin.
+narrateur|La maison de bois craque.
+narrateur|Ça sent le biscuit, tout chaud.
+narrateur|Une vapeur danse près du four.
+narrateur|Dehors, une pierre grise chauffe.
+narrateur|Un oiseau de montagne crie, haut.
 maman|Nino, le biscuit est prêt.
-enfant-m|On le mange dehors ?
+enfant-m|On le mange dehors, tout de suite ?
 maman|Oui, sur la pente.
 maman|Un pique-nique, tout petit.
-narrateur|En ce moment, Nino s'accroupit.
-narrateur|Le sac rouge est par terre.
+narrateur|En ce moment, Nino saisit le paquet.
+narrateur|Le papier est tiède sous les doigts.
+enfant-m|Je le porte, maman.
+enfant-m|Pas besoin du sac.
+narrateur|Il prend aussi la gourde verte.
+narrateur|Elle pique, trop froide.
+enfant-m|Aïe !
+narrateur|Il court vers la porte, les bras pleins.
+narrateur|Le vent pousse le battant.
+narrateur|Le paquet glisse.
+narrateur|La gourde tombe sur le bois.
+narrateur|Patatras.
+enfant-m|Oh.
+narrateur|Le biscuit roule vers le seuil.
+narrateur|Nino le rattrape, les joues chaudes.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+maman|Tu voulais partir tout de suite ?
+enfant-m|Le biscuit va refroidir.
+narrateur|Maman s'accroupit, à sa hauteur.
+maman|Où le biscuit voyage-t-il mieux ?
+enfant-m|Dans mes mains.
+narrateur|Le papier se froisse, trop lâche.
+narrateur|Le sac rouge attend par terre.
 narrateur|La sangle est lisse, un peu froide.
-enfant-m|Il est rouge, maman.
+enfant-m|Il est rouge.
 maman|Oui, c'est le tien.
-maman|Le goûter d'abord, encore chaud.
-narrateur|Nino prend le petit paquet.
-narrateur|Le papier fait un bruit doux.
-narrateur|Ça sent encore le biscuit.
-enfant-m|Je le mange maintenant ?
-maman|Plus tard, dans l'herbe.
-maman|D'abord, dans le sac.
-narrateur|Nino pose le goûter dedans.
-maman|Prends aussi de l'eau.
-narrateur|Nino prend la gourde verte.
-narrateur|Elle est trop froide pour ses doigts.
-enfant-m|Aïe, elle pique.
-maman|Enveloppe-la dans le linge.
-narrateur|Un linge à carreaux attend sur la table.
+narrateur|Nino pose le biscuit dedans.
+narrateur|Le papier se tait.
+maman|L'eau aussi.
+narrateur|Un linge à carreaux attend.
 narrateur|Nino l'enroule autour de l'eau.
-narrateur|Le froid s'en va un peu.
-enfant-m|C'est mieux.
-narrateur|Il pose la gourde dans le sac.
+enfant-m|C'est moins froid.
+narrateur|Il glisse l'eau dans le sac.
 enfant-m|Où est le chapeau ?
 narrateur|Le crochet du bas est vide.
-narrateur|Le chapeau est trop haut.
-maman|Je te le tends ?
-enfant-m|Oui, s'il te plaît.</t>
+narrateur|Le chapeau est trop haut.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>vent,casserole</t>
         </is>
       </c>
     </row>
@@ -1395,12 +1417,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino prépare le sac. Où met-il les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dounia prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Où met-il les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1463,7 +1485,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1471,10 +1493,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1489,11 +1511,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1504,23 +1526,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1529,13 +1551,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1545,7 +1567,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les affaires voyagent dans le sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1578,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maman tend le chapeau. Il est tout mou, un peu chaud. Nino le met dans le sac. Il est dedans. Merci, Nino. Tu as aidé tes doigts aussi. Nino appuie sur la fermeture. Ça fait zzz. Le sac rouge est fermé. Le sac est prêt ? Oui, maman. Nino pose la main sur le rouge. Le papier du goûter se tait. Le biscuit voyage avec nous. Dans le sac. On met tes chaussures ? Oui.</t>
+          <t>Nino pousse une chaise vers le crochet. La chaise glisse sur le bois. Le chapeau penche, trop loin. Je n'arrive pas. Ses épaules baissent. Tu regardes, d'abord ? Nino refuse de foncer. J'attends. Il pose un pied sur la marche. L'éclat de marche accroche la sangle. Nino tire, trop vite. La sangle reste. Ça tient. Maman se tait. Nino observe le sac, puis la marche. Le même éclat pâle, du début. C'est lui. Il soulève la sangle, sans tirer. La sangle passe. Il prend le chapeau, mou, tiède. Il le pose dans le sac. Il est dedans. Merci, Nino. La sangle est libre. Nino appuie sur la fermeture. Ça fait zzz. Le sac rouge est fermé. Le sac est prêt ? Oui, maman. Nino pose la main sur le rouge. Le biscuit voyage avec nous. Dans le sac. On met tes chaussures ? Oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Maman tend le chapeau. Il est tout mou, un peu chaud. Nino le met dans le sac. Il est dedans. Merci, Nino. Tu as aidé tes doigts aussi. Nino appuie sur la fermeture. Ça fait zzz. Le sac rouge est fermé. Le sac est prêt ? Oui, maman. Nino pose la main sur le rouge. Le papier du goûter se tait. Le biscuit voyage avec nous. Dans le sac. On met tes chaussures ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nino pousse une chaise vers le crochet. La chaise glisse sur le bois. Le chapeau penche, trop loin. Je n'arrive pas. Ses épaules baissent. Tu regardes, d'abord ? Nino refuse de foncer. J'attends. Il pose un pied sur la marche. L'éclat de marche accroche la &lt;emphasis level="moderate"&gt;sangle&lt;/emphasis&gt;. Nino tire, trop vite. La sangle reste. Ça tient. Maman se tait. Nino observe le sac, puis la marche. Le même éclat pâle, du début. C'est lui. Il soulève la sangle, sans tirer. La sangle passe. Il prend le chapeau, mou, tiède. Il le pose dans le sac. Il est dedans. Merci, Nino. La sangle est libre. Nino appuie sur la fermeture. Ça fait zzz. Le sac rouge est fermé. Le sac est prêt ? Oui, maman. Nino pose la main sur le rouge. Le biscuit voyage avec nous. Dans le sac. On met tes chaussures ? Oui.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dounia a écouté. Elle a mis la gourde. Elle a mis le chapeau. Elle a mis le goûter. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est prêt. C'est ce que l'adulte a dit.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nino pousse une chaise vers le crochet. La chaise glisse sur le bois. Le chapeau penche, trop loin. Je n'arrive pas. Ses épaules baissent. Tu regardes, d'abord ? Nino refuse de foncer. J'attends. Il pose un pied sur la marche. L'éclat de marche accroche la &lt;emphasis&gt;sangle&lt;/emphasis&gt;. Nino tire, trop vite. La sangle reste. Ça tient. Maman se tait. Nino observe le sac, puis la marche. Le même éclat pâle, du début. C'est lui. Il soulève la sangle, sans tirer. La sangle passe. Il prend le chapeau, mou, tiède. Il le pose dans le sac. Il est dedans. Merci, Nino. La sangle est libre. Nino appuie sur la fermeture. Ça fait zzz. Le sac rouge est fermé. Le sac est prêt ? Oui, maman. Nino pose la main sur le rouge. Le biscuit voyage avec nous. Dans le sac. On met tes chaussures ? Oui.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1635,7 +1657,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1643,22 +1665,26 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE4" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF4" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1669,30 +1695,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>sangle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1701,46 +1727,68 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT4" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=obstacle; intention=ralentir_sans_effrayer; emotion=découragement_léger; intensite=2; destinataire=enfant; sous_texte=l_eclat de marche tient la sangle; tempo=resserré; sourire=aucun; respiration=retenue</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Maman tend le chapeau.
-narrateur|Il est tout mou, un peu chaud.
-narrateur|Nino le met dans le sac.
+          <t>narrateur|Nino pousse une chaise vers le crochet.
+narrateur|La chaise glisse sur le bois.
+narrateur|Le chapeau penche, trop loin.
+enfant-m|Je n'arrive pas.
+narrateur|Ses épaules baissent.
+maman|Tu regardes, d'abord ?
+narrateur|Nino refuse de foncer.
+enfant-m|J'attends.
+narrateur|Il pose un pied sur la marche.
+narrateur|L'éclat de marche accroche la sangle.
+narrateur|Nino tire, trop vite.
+narrateur|La sangle reste.
+enfant-m|Ça tient.
+narrateur|Maman se tait.
+narrateur|Nino observe le sac, puis la marche.
+narrateur|Le même éclat pâle, du début.
+enfant-m|C'est lui.
+narrateur|Il soulève la sangle, sans tirer.
+narrateur|La sangle passe.
+narrateur|Il prend le chapeau, mou, tiède.
+narrateur|Il le pose dans le sac.
 enfant-m|Il est dedans.
 maman|Merci, Nino.
-maman|Tu as aidé tes doigts aussi.
+maman|La sangle est libre.
 narrateur|Nino appuie sur la fermeture.
 narrateur|Ça fait zzz.
 narrateur|Le sac rouge est fermé.
 maman|Le sac est prêt ?
 enfant-m|Oui, maman.
 narrateur|Nino pose la main sur le rouge.
-narrateur|Le papier du goûter se tait.
 maman|Le biscuit voyage avec nous.
 enfant-m|Dans le sac.
 maman|On met tes chaussures ?
 enfant-m|Oui.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1765,17 +1813,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile ses chaussures. La semelle gratte le bois. Tu as fini tes chaussures ? Oui, maman. Maman ouvre la porte. L'air de la pente entre, frais. L'herbe est un peu sèche. Ils s'assoient près d'une pierre chaude. Le goûter, maintenant ? Oui, il est dans le sac. Nino ouvre un tout petit peu. Le papier fait encore un bruit. Une fourmi passe dans l'herbe. Elle veut le biscuit ? Elle a son chemin. Nous, le nôtre. Nino sort le paquet. Le biscuit est encore un peu chaud. Il sent bon. Tu croques ? Oui.</t>
+          <t>Nino enfile ses chaussures. La semelle gratte le bois. Tu as fini tes chaussures ? Oui, maman. Maman ouvre la porte. L'air de la pente entre, frais. L'herbe est un peu sèche. Ils s'assoient près d'une pierre chaude. Le goûter, maintenant ? Oui, il est dans le sac. Nino ouvre un tout petit peu. Le papier fait un bruit fin. Une fourmi passe dans l'herbe. Elle veut le biscuit ? Elle a son chemin. Nous, le nôtre. Nino sort le paquet. Le biscuit est un peu chaud. Il sent bon. Tu croques ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino enfile ses chaussures. La semelle gratte le bois. Tu as fini tes chaussures ? Oui, maman. Maman ouvre la porte. L'air de la pente entre, frais. L'herbe est un peu sèche. Ils s'assoient près d'une pierre chaude. Le goûter, maintenant ? Oui, il est dans le sac. Nino ouvre un tout petit peu. Le papier fait encore un bruit. Une fourmi passe dans l'herbe. Elle veut le biscuit ? Elle a son chemin. Nous, le nôtre. Nino sort le paquet. Le biscuit est encore un peu chaud. Il sent bon. Tu croques ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino enfile ses chaussures. La semelle gratte le bois. Tu as fini tes chaussures ? Oui, maman. Maman ouvre la porte. L'air de la pente entre, frais. L'herbe est un peu sèche. Ils s'assoient près d'une pierre chaude. Le goûter, maintenant ? Oui, il est dans le sac. Nino ouvre un tout petit peu. Le papier fait un bruit fin. Une fourmi passe dans l'herbe. Elle veut le &lt;emphasis level="moderate"&gt;biscuit&lt;/emphasis&gt; ? Elle a son chemin. Nous, le nôtre. Nino sort le paquet. Le biscuit est un peu chaud. Il sent bon. Tu croques ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Dounia prend le &lt;emphasis&gt;sac&lt;/emphasis&gt;. La sangle est lisse. Maman ouvre la porte. Elles partent.&lt;/slow&gt; [pause]</t>
+          <t>Nino enfile ses chaussures. La semelle gratte le bois. Tu as fini tes chaussures ? Oui, maman. Maman ouvre la porte. L'air de la pente entre, frais. L'herbe est un peu sèche. Ils s'assoient près d'une pierre chaude. Le goûter, maintenant ? Oui, il est dans le sac. Nino ouvre un tout petit peu. Le papier fait un bruit fin. Une fourmi passe dans l'herbe. Elle veut le &lt;emphasis&gt;biscuit&lt;/emphasis&gt; ? Elle a son chemin. Nous, le nôtre. Nino sort le paquet. Le biscuit est un peu chaud. Il sent bon. Tu croques ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1870,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,10 +1878,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,30 +1904,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>biscuit</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,10 +1936,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1900,9 +1948,13 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=mener_au_pique_nique; emotion=élan_retenu; intensite=2; destinataire=enfant; sous_texte=le biscuit attend dans le sac; tempo=vif; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Nino enfile ses chaussures.
@@ -1916,18 +1968,23 @@
 enfant-m|Le goûter, maintenant ?
 maman|Oui, il est dans le sac.
 narrateur|Nino ouvre un tout petit peu.
-narrateur|Le papier fait encore un bruit.
+narrateur|Le papier fait un bruit fin.
 narrateur|Une fourmi passe dans l'herbe.
 enfant-m|Elle veut le biscuit ?
 maman|Elle a son chemin.
 maman|Nous, le nôtre.
 narrateur|Nino sort le paquet.
-narrateur|Le biscuit est encore un peu chaud.
+narrateur|Le biscuit est un peu chaud.
 enfant-m|Il sent bon.
 maman|Tu croques ?
 enfant-m|Oui.</t>
         </is>
       </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>herbe,vent</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1952,17 +2009,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Nino croque le biscuit. La croûte casse, toute légère. Il est encore chaud. Comme le four, tout à l'heure. Le sac rouge repose dans l'herbe. Le vent de la pente passe encore. Le biscuit est encore tout chaud. La pierre grise reste chaude sous la main.</t>
+          <t>Nino croque le biscuit. La croûte casse, toute légère. Il est chaud. Comme le four, à l'instant. Le sac rouge repose dans l'herbe. Le vent de la pente passe. La pierre grise chauffe sous la main. Sur le rouge, un éclat de marche. Il a voyagé aussi. Oui. Le même, pâle, minuscule.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Nino croque le biscuit. La croûte casse, toute légère. Il est encore chaud. Comme le four, tout à l'heure. Le sac rouge repose dans l'herbe. Le vent de la pente passe encore. Le biscuit est encore tout chaud. La pierre grise reste chaude sous la main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino croque le biscuit. La croûte casse, toute légère. Il est chaud. Comme le four, à l'instant. Le sac rouge repose dans l'herbe. Le vent de la pente passe. La pierre grise chauffe sous la main. Sur le rouge, un &lt;emphasis level="moderate"&gt;éclat de marche&lt;/emphasis&gt;. Il a voyagé aussi. Oui. Le même, pâle, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino croque le biscuit. La croûte casse, toute légère. Il est chaud. Comme le four, à l'instant. Le sac rouge repose dans l'herbe. Le vent de la pente passe. La pierre grise chauffe sous la main. Sur le rouge, un &lt;emphasis&gt;éclat de marche&lt;/emphasis&gt;. Il a voyagé aussi. Oui. Le même, pâle, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,18 +2066,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2029,12 +2086,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2100,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de marche</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2123,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,31 +2136,38 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat de marche a voyagé sur le sac; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Nino croque le biscuit.
 narrateur|La croûte casse, toute légère.
-enfant-m|Il est encore chaud.
-maman|Comme le four, tout à l'heure.
+enfant-m|Il est chaud.
+maman|Comme le four, à l'instant.
 narrateur|Le sac rouge repose dans l'herbe.
-narrateur|Le vent de la pente passe encore.
-maman|Le biscuit est encore tout chaud.
-narrateur|La pierre grise reste chaude sous la main.</t>
+narrateur|Le vent de la pente passe.
+narrateur|La pierre grise chauffe sous la main.
+narrateur|Sur le rouge, un éclat de marche.
+enfant-m|Il a voyagé aussi.
+maman|Oui.
+narrateur|Le même, pâle, minuscule.</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2184,6 +2252,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>